<commit_message>
Set swl_slr to 0 in example inputs and PSE templates
The 176.45 m value double-added the Chicago datum: CHS-GLM storm databases
already store water levels in IGLD85.
</commit_message>
<xml_diff>
--- a/CHESS_Library/PSE_Templates/floodwall_pse.xlsx
+++ b/CHESS_Library/PSE_Templates/floodwall_pse.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0_StormSim_Task\StormSim-Library\CHESS_Library\PSE_Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0_StormSim_Task\CHESS-Library\CHESS_Library\PSE_Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{191F2631-E154-4218-8B4F-DB4D79794798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AAE2B5-C1E4-4EAD-921C-AA28074FA979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="25305" windowHeight="20985" xr2:uid="{DC0F9EFB-6E2F-481A-B00B-37B31DD1708E}"/>
+    <workbookView xWindow="4635" yWindow="4635" windowWidth="28800" windowHeight="15270" xr2:uid="{DC0F9EFB-6E2F-481A-B00B-37B31DD1708E}"/>
   </bookViews>
   <sheets>
     <sheet name="floodwall_pse" sheetId="1" r:id="rId1"/>
@@ -1835,7 +1835,7 @@
         <v>47</v>
       </c>
       <c r="D12" s="18">
-        <v>176.45</v>
+        <v>0</v>
       </c>
       <c r="F12" s="20"/>
       <c r="G12" s="20"/>

</xml_diff>

<commit_message>
templates: drop toe_elevation from floodwall templates
Floodwall toes always come from wall_bottom_elevation at run time.
</commit_message>
<xml_diff>
--- a/CHESS_Library/PSE_Templates/floodwall_pse.xlsx
+++ b/CHESS_Library/PSE_Templates/floodwall_pse.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0_StormSim_Task\CHESS-Library\CHESS_Library\PSE_Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3AAE2B5-C1E4-4EAD-921C-AA28074FA979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C3C06BE-BF39-4275-A941-924762B53ADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4635" yWindow="4635" windowWidth="28800" windowHeight="15270" xr2:uid="{DC0F9EFB-6E2F-481A-B00B-37B31DD1708E}"/>
+    <workbookView xWindow="5670" yWindow="5610" windowWidth="28800" windowHeight="15270" xr2:uid="{DC0F9EFB-6E2F-481A-B00B-37B31DD1708E}"/>
   </bookViews>
   <sheets>
     <sheet name="floodwall_pse" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="116">
   <si>
     <t>CHESS Project General Inputs</t>
   </si>
@@ -287,12 +287,6 @@
   </si>
   <si>
     <t>Crest Width/Wall Width</t>
-  </si>
-  <si>
-    <t>toe_elevation</t>
-  </si>
-  <si>
-    <t>Mound Toe Elevation (Negative Below Datum Zero)</t>
   </si>
   <si>
     <t>wall_bottom_elevation</t>
@@ -1557,7 +1551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{575F4332-2D16-4B46-9F46-3F3DF76F4165}">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="63.85546875" bestFit="1" customWidth="1"/>
@@ -2147,7 +2141,7 @@
         <v>47</v>
       </c>
       <c r="D33" s="9">
-        <v>176.2</v>
+        <v>175.8</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -2158,122 +2152,122 @@
         <v>92</v>
       </c>
       <c r="C34" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B35" t="s">
+        <v>94</v>
+      </c>
+      <c r="C35" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D34" s="9">
-        <v>175.8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="35" t="s">
-        <v>93</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D35" s="9">
-        <v>8</v>
+      <c r="D35" s="10">
+        <v>173.99</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="33"/>
+      <c r="B36" s="33"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+    </row>
+    <row r="37" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+    </row>
+    <row r="38" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="C36" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D36" s="10">
-        <v>173.99</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="33"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="33"/>
-      <c r="D37" s="33"/>
-    </row>
-    <row r="38" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="36" t="s">
+      <c r="B39" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="B38" s="37"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="37"/>
-    </row>
-    <row r="39" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="5" t="s">
+      <c r="C39" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="D39" s="18">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="360.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="C40" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="39">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="37"/>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
+    </row>
+    <row r="42" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="B42" s="41"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="41"/>
+    </row>
+    <row r="43" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B43" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C43" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="D43" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="B40" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="C40" s="17" t="s">
-        <v>100</v>
-      </c>
-      <c r="D40" s="18">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="360.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="B41" s="38" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="C41" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D41" s="39">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="37"/>
-      <c r="B42" s="37"/>
-      <c r="C42" s="37"/>
-      <c r="D42" s="37"/>
-    </row>
-    <row r="43" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="40" t="s">
+      <c r="B44" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="B43" s="41"/>
-      <c r="C43" s="41"/>
-      <c r="D43" s="41"/>
-    </row>
-    <row r="44" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>5</v>
+      <c r="C44" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="18">
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -2301,7 +2295,7 @@
         <v>9</v>
       </c>
       <c r="D46" s="18">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -2315,7 +2309,7 @@
         <v>9</v>
       </c>
       <c r="D47" s="18">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -2346,31 +2340,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="15" t="s">
+    <row r="50" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="B50" s="16" t="s">
+      <c r="B50" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="C50" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D50" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="B51" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="C51" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D51" s="24">
+      <c r="C50" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D50" s="24">
         <v>1</v>
       </c>
     </row>

</xml_diff>